<commit_message>
adding modified templates to match new evidence link coulumn
</commit_message>
<xml_diff>
--- a/examples/starters/uofa-starter-filled.xlsx
+++ b/examples/starters/uofa-starter-filled.xlsx
@@ -35,7 +35,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -131,8 +131,19 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00666666"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -169,8 +180,18 @@
         <bgColor rgb="FFF2F3F4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001B4F72"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F3F4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -193,6 +214,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -204,7 +239,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -311,6 +346,12 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -768,7 +809,7 @@
           <t>https://windtech.com/reports/blade-fatigue-2026</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L4" s="17" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -973,7 +1014,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="18">
@@ -1032,7 +1073,7 @@
           <t>Decision Outcome</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="17" t="inlineStr">
         <is>
           <t>Has UQ (COU-level)</t>
         </is>
@@ -1092,7 +1133,7 @@
           <t>Accepted</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L2" s="17" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1152,7 +1193,7 @@
           <t>Not accepted</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L3" s="17" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1227,7 +1268,7 @@
       <c r="I5" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J5" s="17" t="inlineStr">
         <is>
           <t>not-applicable</t>
         </is>
@@ -1244,7 +1285,7 @@
           <t>MRL 5</t>
         </is>
       </c>
-      <c r="I6" t="n">
+      <c r="I6" s="17" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1276,7 +1317,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1876,7 +1916,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="42" customWidth="1" style="17" min="1" max="1"/>
@@ -1884,6 +1924,7 @@
     <col width="16" customWidth="1" style="17" min="3" max="4"/>
     <col width="40" customWidth="1" style="17" min="5" max="5"/>
     <col width="12" customWidth="1" style="17" min="6" max="6"/>
+    <col width="22" customWidth="1" style="18" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="18">
@@ -1936,6 +1977,11 @@
           <t>Factor Status</t>
         </is>
       </c>
+      <c r="H3" s="37" t="inlineStr">
+        <is>
+          <t>Linked Evidence</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="22.35" customHeight="1" s="18">
       <c r="A4" s="22" t="inlineStr">
@@ -1971,6 +2017,11 @@
       <c r="G4" s="22" t="inlineStr">
         <is>
           <t>assessed / not-assessed / scoped-out / not-applicable</t>
+        </is>
+      </c>
+      <c r="H4" s="38" t="inlineStr">
+        <is>
+          <t>URI of validation result that supports this factor (optional)</t>
         </is>
       </c>
     </row>

</xml_diff>